<commit_message>
Testing with console response
</commit_message>
<xml_diff>
--- a/TestKit/Q1/Header.xlsx
+++ b/TestKit/Q1/Header.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5BBD967-CA9F-407B-ACD7-4C9B95E30B25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF1FCC2C-32F0-4195-83EC-66AFA4C99E80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DataPattern" sheetId="3" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t>Data Type</t>
   </si>
@@ -55,9 +55,6 @@
     <t>TC1</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>TC2_Send</t>
   </si>
   <si>
@@ -89,6 +86,12 @@
   </si>
   <si>
     <t>TCP</t>
+  </si>
+  <si>
+    <t>Grade_Content</t>
+  </si>
+  <si>
+    <t>Client</t>
   </si>
 </sst>
 </file>
@@ -99,7 +102,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -459,14 +462,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" customWidth="1"/>
-    <col min="2" max="2" width="22.21875" customWidth="1"/>
-    <col min="3" max="3" width="21.88671875" customWidth="1"/>
+    <col min="1" max="1" width="18.296875" customWidth="1"/>
+    <col min="2" max="2" width="22.19921875" customWidth="1"/>
+    <col min="3" max="3" width="21.8984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -474,7 +477,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -491,12 +494,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="5" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>4</v>
       </c>
@@ -504,7 +507,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -512,25 +515,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5">
         <v>2</v>
@@ -544,20 +547,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="44.33203125" style="5" customWidth="1"/>
-    <col min="3" max="5" width="8.88671875" style="5" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="1" width="10.69921875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="44.296875" style="5" customWidth="1"/>
+    <col min="3" max="5" width="8.8984375" style="5" customWidth="1"/>
+    <col min="6" max="16384" width="8.8984375" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>11</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -570,7 +573,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" s="5">
         <v>1</v>
@@ -578,7 +581,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" s="5">
         <v>1</v>
@@ -586,7 +589,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5" s="5">
         <v>2</v>
@@ -600,34 +603,43 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9C6C48B-55C0-4A7D-A267-4474B31A4631}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="5" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="4" t="s">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>17</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>